<commit_message>
ccd paper and prospectus revisions
</commit_message>
<xml_diff>
--- a/prosp_draft_data_03_24_github_version.xlsx
+++ b/prosp_draft_data_03_24_github_version.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kom11/Documents/GitHub/phd/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ED70F8C3-C35E-974A-96C2-F112AECC5472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A133B8-4F1E-974E-BBB1-5ADCE8729585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15500" yWindow="-28200" windowWidth="29700" windowHeight="28200" xr2:uid="{C3B414E7-4F74-B640-BD11-B6FEEAE78456}"/>
+    <workbookView xWindow="4500" yWindow="900" windowWidth="29700" windowHeight="21000" xr2:uid="{C3B414E7-4F74-B640-BD11-B6FEEAE78456}"/>
   </bookViews>
   <sheets>
     <sheet name="drafting database" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="4" r:id="rId2"/>
+    <sheet name="Level of Rule" sheetId="4" r:id="rId2"/>
     <sheet name="state_poverty_by_race" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="283">
   <si>
     <t>state</t>
   </si>
@@ -983,6 +983,45 @@
   </si>
   <si>
     <t>PID</t>
+  </si>
+  <si>
+    <t>Constitutional</t>
+  </si>
+  <si>
+    <t>Statutory</t>
+  </si>
+  <si>
+    <t>Administrative</t>
+  </si>
+  <si>
+    <t>Combination</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Chamber</t>
+  </si>
+  <si>
+    <t>House</t>
+  </si>
+  <si>
+    <t>Senate</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Categorical </t>
+  </si>
+  <si>
+    <t>Offense-Specific</t>
+  </si>
+  <si>
+    <t>Conditioning Policies</t>
+  </si>
+  <si>
+    <t>Permanent/Tempoarary</t>
   </si>
 </sst>
 </file>
@@ -1179,7 +1218,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1359,6 +1398,24 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -1521,7 +1578,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1544,10 +1601,13 @@
     <xf numFmtId="2" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1967,24 +2027,24 @@
       </c>
       <c r="N1" s="9"/>
       <c r="O1" s="9"/>
-      <c r="P1" s="8" t="s">
+      <c r="P1" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="Q1" s="8"/>
-      <c r="R1" s="8"/>
-      <c r="S1" s="8"/>
-      <c r="T1" s="8"/>
-      <c r="U1" s="8"/>
-      <c r="V1" s="8"/>
-      <c r="W1" s="8"/>
-      <c r="X1" s="8"/>
-      <c r="Y1" s="8"/>
-      <c r="Z1" s="8"/>
-      <c r="AA1" s="8"/>
-      <c r="AB1" s="8"/>
-      <c r="AC1" s="8"/>
-      <c r="AD1" s="8"/>
-      <c r="AE1" s="8"/>
+      <c r="Q1" s="10"/>
+      <c r="R1" s="10"/>
+      <c r="S1" s="10"/>
+      <c r="T1" s="10"/>
+      <c r="U1" s="10"/>
+      <c r="V1" s="10"/>
+      <c r="W1" s="10"/>
+      <c r="X1" s="10"/>
+      <c r="Y1" s="10"/>
+      <c r="Z1" s="10"/>
+      <c r="AA1" s="10"/>
+      <c r="AB1" s="10"/>
+      <c r="AC1" s="10"/>
+      <c r="AD1" s="10"/>
+      <c r="AE1" s="10"/>
     </row>
     <row r="2" spans="1:79" ht="159" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
@@ -2284,7 +2344,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="7" spans="1:79" ht="238" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:79" ht="170" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>40</v>
       </c>
@@ -2335,7 +2395,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="8" spans="1:79" ht="323" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:79" ht="238" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>41</v>
       </c>
@@ -2355,7 +2415,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="9" spans="1:79" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:79" ht="356" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>42</v>
       </c>
@@ -2454,7 +2514,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="15" spans="1:79" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:79" ht="323" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>48</v>
       </c>
@@ -2471,7 +2531,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="16" spans="1:79" ht="356" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:79" ht="255" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>49</v>
       </c>
@@ -2488,7 +2548,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="17" spans="1:66" ht="289" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:66" ht="221" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>50</v>
       </c>
@@ -2525,7 +2585,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="19" spans="1:66" ht="272" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:66" ht="204" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>52</v>
       </c>
@@ -2542,7 +2602,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="20" spans="1:66" ht="68" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:66" ht="51" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>53</v>
       </c>
@@ -2579,7 +2639,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="22" spans="1:66" ht="204" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:66" ht="136" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>55</v>
       </c>
@@ -2616,7 +2676,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="24" spans="1:66" ht="136" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:66" ht="102" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>57</v>
       </c>
@@ -2673,7 +2733,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="27" spans="1:66" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:66" ht="372" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>60</v>
       </c>
@@ -2690,7 +2750,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="28" spans="1:66" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:66" ht="388" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>61</v>
       </c>
@@ -2710,7 +2770,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="29" spans="1:66" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:66" ht="340" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>62</v>
       </c>
@@ -2727,7 +2787,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="30" spans="1:66" ht="34" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:66" ht="17" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>63</v>
       </c>
@@ -2744,7 +2804,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="31" spans="1:66" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:66" ht="404" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>64</v>
       </c>
@@ -2861,7 +2921,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="37" spans="1:68" ht="204" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:68" ht="153" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>70</v>
       </c>
@@ -2952,7 +3012,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="42" spans="1:68" ht="255" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:68" ht="204" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>75</v>
       </c>
@@ -2975,7 +3035,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="43" spans="1:68" ht="340" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:68" ht="272" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>76</v>
       </c>
@@ -3023,7 +3083,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="46" spans="1:68" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:68" ht="372" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>79</v>
       </c>
@@ -3063,7 +3123,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="48" spans="1:68" ht="238" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:68" ht="170" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>81</v>
       </c>
@@ -3094,7 +3154,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="50" spans="1:66" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:66" ht="372" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>83</v>
       </c>
@@ -3253,9 +3313,868 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07317766-2635-6C4C-99D4-940F0F196B90}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:M103"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.5" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="10" max="10" width="15.6640625" customWidth="1"/>
+    <col min="12" max="12" width="18.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="B1" t="s">
+        <v>275</v>
+      </c>
+      <c r="C1" t="s">
+        <v>270</v>
+      </c>
+      <c r="D1" t="s">
+        <v>271</v>
+      </c>
+      <c r="E1" t="s">
+        <v>272</v>
+      </c>
+      <c r="F1" t="s">
+        <v>273</v>
+      </c>
+      <c r="G1" t="s">
+        <v>274</v>
+      </c>
+      <c r="I1" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" t="s">
+        <v>280</v>
+      </c>
+      <c r="L1" t="s">
+        <v>282</v>
+      </c>
+      <c r="M1" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="34" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="34" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B19" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B24" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B27" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B28" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B32" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B34" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B35" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B36" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B37" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B38" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B39" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B40" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B42" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B43" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B44" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B45" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B46" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B47" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B48" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B49" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B50" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B51" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B52" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B53" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>63</v>
+      </c>
+      <c r="B54" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>63</v>
+      </c>
+      <c r="B55" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>64</v>
+      </c>
+      <c r="B56" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>64</v>
+      </c>
+      <c r="B57" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>65</v>
+      </c>
+      <c r="B58" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>65</v>
+      </c>
+      <c r="B59" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>66</v>
+      </c>
+      <c r="B60" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>66</v>
+      </c>
+      <c r="B61" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>67</v>
+      </c>
+      <c r="B62" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>67</v>
+      </c>
+      <c r="B63" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>68</v>
+      </c>
+      <c r="B64" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>68</v>
+      </c>
+      <c r="B65" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>69</v>
+      </c>
+      <c r="B66" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>70</v>
+      </c>
+      <c r="B68" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>70</v>
+      </c>
+      <c r="B69" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>71</v>
+      </c>
+      <c r="B70" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>71</v>
+      </c>
+      <c r="B71" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>72</v>
+      </c>
+      <c r="B72" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>73</v>
+      </c>
+      <c r="B75" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>74</v>
+      </c>
+      <c r="B76" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>74</v>
+      </c>
+      <c r="B77" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>75</v>
+      </c>
+      <c r="B78" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>75</v>
+      </c>
+      <c r="B79" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>76</v>
+      </c>
+      <c r="B80" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>76</v>
+      </c>
+      <c r="B81" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>77</v>
+      </c>
+      <c r="B82" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>77</v>
+      </c>
+      <c r="B83" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>78</v>
+      </c>
+      <c r="B84" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>78</v>
+      </c>
+      <c r="B85" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>79</v>
+      </c>
+      <c r="B86" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>79</v>
+      </c>
+      <c r="B87" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>80</v>
+      </c>
+      <c r="B88" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>80</v>
+      </c>
+      <c r="B89" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>81</v>
+      </c>
+      <c r="B90" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>81</v>
+      </c>
+      <c r="B91" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>82</v>
+      </c>
+      <c r="B92" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>82</v>
+      </c>
+      <c r="B93" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>83</v>
+      </c>
+      <c r="B94" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>83</v>
+      </c>
+      <c r="B95" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>84</v>
+      </c>
+      <c r="B96" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>84</v>
+      </c>
+      <c r="B97" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>85</v>
+      </c>
+      <c r="B98" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>85</v>
+      </c>
+      <c r="B99" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>86</v>
+      </c>
+      <c r="B100" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>86</v>
+      </c>
+      <c r="B101" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>87</v>
+      </c>
+      <c r="B102" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
+        <v>87</v>
+      </c>
+      <c r="B103" t="s">
+        <v>277</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>